<commit_message>
Updated KiCad and Parts list for new SD Card Slot
Updated KiCad schematic, PCB, and parts list for new SD card slot Molex 5033981892
</commit_message>
<xml_diff>
--- a/KiCad_files/MusselGapeTracker_RevI/MusselGapeTracker_RevI_parts_list.xlsx
+++ b/KiCad_files/MusselGapeTracker_RevI/MusselGapeTracker_RevI_parts_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/Documents/GitHub/MusselGapeTracker_hardware/KiCad_files/MusselGapeTracker_RevI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D78DAA-E179-4C42-B825-35288CA3C3B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43077F51-7C1D-624E-9A16-CF8452D05F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MusselGapeTracker_RevH" sheetId="2" r:id="rId1"/>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="439">
   <si>
     <t>Part Description</t>
   </si>
@@ -396,9 +396,6 @@
     <t>miller.lbr\MICROSD_MOLEX_REVERSECURRENT</t>
   </si>
   <si>
-    <t>MicroSD card slot push-push</t>
-  </si>
-  <si>
     <t>miller.lbr\ATMEGA328_SMT</t>
   </si>
   <si>
@@ -1326,9 +1323,6 @@
     <t>https://oshpark.com/shared_projects/NMAsMegv</t>
   </si>
   <si>
-    <t>MusselGapeTracker RevH stencil</t>
-  </si>
-  <si>
     <t>Hall effect sensor board stencil</t>
   </si>
   <si>
@@ -1372,15 +1366,6 @@
   </si>
   <si>
     <t>NEED SUB IF USING DIFF HEADER</t>
-  </si>
-  <si>
-    <t>GCT</t>
-  </si>
-  <si>
-    <t>MEM2052-00-195-00-A</t>
-  </si>
-  <si>
-    <t>2073-MEM2052-00-195-00-ACT-ND</t>
   </si>
   <si>
     <t>slater substitute alt for main</t>
@@ -1417,7 +1402,16 @@
     <t>^/ft</t>
   </si>
   <si>
-    <t>MusselGapeTracker_RevI_circuit board (order of 3)</t>
+    <t>MusselGapeTracker RevI stencil</t>
+  </si>
+  <si>
+    <t>MusselGapeTracker_RevI circuit board (order of 3)</t>
+  </si>
+  <si>
+    <t>MicroSD card slot 5033981892</t>
+  </si>
+  <si>
+    <t>WM11190CT-ND</t>
   </si>
 </sst>
 </file>
@@ -2058,7 +2052,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="15" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -2087,19 +2081,19 @@
         <v>12</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="J2" s="15" t="s">
+        <v>337</v>
+      </c>
+      <c r="K2" s="15" t="s">
         <v>338</v>
       </c>
-      <c r="K2" s="15" t="s">
-        <v>339</v>
-      </c>
       <c r="L2" s="15" t="s">
+        <v>341</v>
+      </c>
+      <c r="M2" s="15" t="s">
         <v>342</v>
-      </c>
-      <c r="M2" s="15" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="32" x14ac:dyDescent="0.2">
@@ -2158,7 +2152,7 @@
     </row>
     <row r="5" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -2167,13 +2161,13 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E5" s="7">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G5" s="6">
         <v>0.73</v>
@@ -2185,7 +2179,7 @@
     </row>
     <row r="6" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="40" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
@@ -2194,13 +2188,13 @@
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="E6" s="7">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="G6" s="6">
         <v>0.65</v>
@@ -2210,7 +2204,7 @@
         <v>0.65</v>
       </c>
       <c r="I6" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
@@ -2242,7 +2236,7 @@
     </row>
     <row r="8" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
@@ -2251,13 +2245,13 @@
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E8" s="7">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G8" s="6">
         <v>0.1</v>
@@ -2404,22 +2398,22 @@
     </row>
     <row r="14" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B14" t="s">
         <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D14" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E14" s="7">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G14" s="6">
         <v>0.62</v>
@@ -2429,16 +2423,16 @@
         <v>0.62</v>
       </c>
       <c r="J14" t="s">
+        <v>339</v>
+      </c>
+      <c r="K14" t="s">
         <v>340</v>
       </c>
-      <c r="K14" t="s">
-        <v>341</v>
-      </c>
       <c r="L14" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="M14" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="16" x14ac:dyDescent="0.2">
@@ -2470,7 +2464,7 @@
     </row>
     <row r="16" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B16" t="s">
         <v>46</v>
@@ -2479,13 +2473,13 @@
         <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E16" s="7">
         <v>16</v>
       </c>
       <c r="F16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G16" s="6">
         <v>1.22</v>
@@ -2497,19 +2491,19 @@
     </row>
     <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C17" t="s">
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E17" s="7">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G17" s="6">
         <v>12.46</v>
@@ -2519,10 +2513,10 @@
         <v>12.46</v>
       </c>
       <c r="J17" t="s">
+        <v>407</v>
+      </c>
+      <c r="K17" t="s">
         <v>408</v>
-      </c>
-      <c r="K17" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2560,13 +2554,13 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E19" s="7">
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G19" s="6">
         <v>1.03</v>
@@ -2603,7 +2597,7 @@
         <v>3.84</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2630,7 +2624,7 @@
         <v>1.6</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2658,10 +2652,10 @@
       </c>
       <c r="I22" s="39"/>
       <c r="J22" t="s">
+        <v>349</v>
+      </c>
+      <c r="K22" t="s">
         <v>350</v>
-      </c>
-      <c r="K22" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2771,7 +2765,7 @@
     </row>
     <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B27" t="s">
         <v>92</v>
@@ -2796,30 +2790,30 @@
         <v>0.51</v>
       </c>
       <c r="J27" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K27" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="40" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="B28" t="s">
         <v>95</v>
       </c>
       <c r="C28" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="D28" t="s">
+        <v>345</v>
+      </c>
+      <c r="E28" s="7">
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
         <v>346</v>
-      </c>
-      <c r="E28" s="7">
-        <v>1</v>
-      </c>
-      <c r="F28" t="s">
-        <v>347</v>
       </c>
       <c r="G28" s="6">
         <v>0.42</v>
@@ -2829,7 +2823,7 @@
         <v>0.42</v>
       </c>
       <c r="I28" s="41" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="J28" t="s">
         <v>96</v>
@@ -2855,7 +2849,7 @@
         <v>2</v>
       </c>
       <c r="F29" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G29" s="6">
         <v>0.72</v>
@@ -2867,49 +2861,49 @@
     </row>
     <row r="30" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="40" t="s">
-        <v>103</v>
+        <v>437</v>
       </c>
       <c r="B30" t="s">
         <v>102</v>
       </c>
       <c r="C30" t="s">
-        <v>429</v>
-      </c>
-      <c r="D30" t="s">
-        <v>430</v>
+        <v>72</v>
+      </c>
+      <c r="D30">
+        <v>5033981892</v>
       </c>
       <c r="E30" s="7">
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="G30" s="6">
-        <v>1.1200000000000001</v>
+        <v>2.62</v>
       </c>
       <c r="H30" s="6">
         <f t="shared" si="0"/>
-        <v>1.1200000000000001</v>
+        <v>2.62</v>
       </c>
       <c r="I30" s="41" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="37" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C31" t="s">
         <v>101</v>
       </c>
       <c r="D31" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="E31" s="7">
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="G31" s="6">
         <v>1.25</v>
@@ -2919,27 +2913,27 @@
         <v>1.25</v>
       </c>
       <c r="I31" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B32" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C32" t="s">
         <v>93</v>
       </c>
       <c r="D32" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E32" s="7">
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G32" s="6">
         <v>2.74</v>
@@ -2949,18 +2943,18 @@
         <v>2.74</v>
       </c>
       <c r="J32" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="K32" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" t="s">
         <v>122</v>
-      </c>
-      <c r="C33" t="s">
-        <v>123</v>
       </c>
       <c r="D33">
         <v>8195</v>
@@ -2969,7 +2963,7 @@
         <v>16</v>
       </c>
       <c r="F33" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G33" s="6">
         <v>0.18</v>
@@ -2981,22 +2975,22 @@
     </row>
     <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B34" t="s">
+        <v>124</v>
+      </c>
+      <c r="C34" t="s">
         <v>125</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>126</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" s="7">
+        <v>1</v>
+      </c>
+      <c r="F34" t="s">
         <v>127</v>
-      </c>
-      <c r="E34" s="7">
-        <v>1</v>
-      </c>
-      <c r="F34" t="s">
-        <v>128</v>
       </c>
       <c r="G34" s="6">
         <v>0.75</v>
@@ -3008,19 +3002,19 @@
     </row>
     <row r="35" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C35" t="s">
+        <v>308</v>
+      </c>
+      <c r="D35" t="s">
         <v>312</v>
       </c>
-      <c r="C35" t="s">
-        <v>309</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="E35" s="7">
+        <v>1</v>
+      </c>
+      <c r="F35" t="s">
         <v>313</v>
-      </c>
-      <c r="E35" s="7">
-        <v>1</v>
-      </c>
-      <c r="F35" t="s">
-        <v>314</v>
       </c>
       <c r="G35" s="6">
         <v>1.71</v>
@@ -3032,22 +3026,22 @@
     </row>
     <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C36" t="s">
         <v>60</v>
       </c>
       <c r="D36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E36" s="7">
         <v>1</v>
       </c>
       <c r="F36" s="22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G36" s="6">
         <v>0.64</v>
@@ -3059,19 +3053,19 @@
     </row>
     <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B37" t="s">
         <v>284</v>
       </c>
-      <c r="B37" t="s">
+      <c r="D37" s="21" t="s">
         <v>285</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="E37" s="7">
+        <v>1</v>
+      </c>
+      <c r="F37" s="21" t="s">
         <v>286</v>
-      </c>
-      <c r="E37" s="7">
-        <v>1</v>
-      </c>
-      <c r="F37" s="21" t="s">
-        <v>287</v>
       </c>
       <c r="G37" s="6">
         <v>0.67</v>
@@ -3108,7 +3102,7 @@
         <v>0.16</v>
       </c>
       <c r="I38" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3135,7 +3129,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="I39" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3162,7 +3156,7 @@
         <v>1.5</v>
       </c>
       <c r="I40" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
@@ -3171,36 +3165,36 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G42" s="19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H42" s="19">
         <f>SUM(H3:H37)</f>
-        <v>70.189999999999984</v>
+        <v>71.689999999999969</v>
       </c>
       <c r="I42" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="40" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C44" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D44" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="E44" s="7">
         <v>72</v>
       </c>
       <c r="F44" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="G44" s="12">
         <v>0.26</v>
@@ -3210,30 +3204,30 @@
         <v>18.72</v>
       </c>
       <c r="I44" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E45" s="7" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="G45" s="42" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="H45" s="12"/>
     </row>
     <row r="54" spans="1:11" ht="30.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="56" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E57" s="7">
         <v>1</v>
@@ -3246,15 +3240,15 @@
         <v>15.066666666666668</v>
       </c>
       <c r="I57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="C58" s="23" t="s">
         <v>410</v>
-      </c>
-      <c r="C58" s="23" t="s">
-        <v>411</v>
       </c>
       <c r="E58" s="7">
         <v>16</v>
@@ -3275,16 +3269,16 @@
     </row>
     <row r="60" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G60" s="11"/>
     </row>
     <row r="61" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>413</v>
+        <v>435</v>
       </c>
       <c r="C61" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E61" s="7">
         <v>1</v>
@@ -3297,15 +3291,15 @@
         <v>0</v>
       </c>
       <c r="I61" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="C62" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E62" s="7">
         <v>1</v>
@@ -3318,22 +3312,22 @@
     </row>
     <row r="64" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E64"/>
       <c r="F64" s="9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="E65" s="7">
+        <v>1</v>
+      </c>
+      <c r="F65" s="36" t="s">
         <v>400</v>
-      </c>
-      <c r="E65" s="7">
-        <v>1</v>
-      </c>
-      <c r="F65" s="36" t="s">
-        <v>401</v>
       </c>
       <c r="G65" s="6">
         <v>9.99</v>
@@ -3345,13 +3339,13 @@
     </row>
     <row r="66" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E66" s="7">
         <v>1</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G66" s="6">
         <v>6.99</v>
@@ -3369,28 +3363,28 @@
       <c r="A68"/>
       <c r="E68"/>
       <c r="G68" s="19" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(H44:H66,H3:H37)</f>
-        <v>128.95666666666665</v>
+        <v>130.45666666666665</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="20" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E69"/>
     </row>
     <row r="70" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
+        <v>106</v>
+      </c>
+      <c r="E70" s="7">
+        <v>1</v>
+      </c>
+      <c r="F70" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="E70" s="7">
-        <v>1</v>
-      </c>
-      <c r="F70" s="4" t="s">
-        <v>108</v>
       </c>
       <c r="G70" s="6">
         <v>44.22</v>
@@ -3400,47 +3394,47 @@
         <v>0</v>
       </c>
       <c r="I70" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C71" t="s">
+        <v>332</v>
+      </c>
+      <c r="D71" t="s">
         <v>333</v>
       </c>
-      <c r="D71" t="s">
-        <v>334</v>
-      </c>
       <c r="E71" s="7">
         <v>1</v>
       </c>
       <c r="F71" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G71" s="6">
         <v>64.5</v>
       </c>
       <c r="I71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C72" t="s">
+        <v>334</v>
+      </c>
+      <c r="D72" t="s">
         <v>335</v>
       </c>
-      <c r="D72" t="s">
-        <v>336</v>
-      </c>
       <c r="E72" s="7">
         <v>1</v>
       </c>
       <c r="F72" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G72" s="6">
         <v>129.94999999999999</v>
@@ -3448,19 +3442,19 @@
     </row>
     <row r="73" spans="1:9" ht="17" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C73" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D73" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E73" s="7">
         <v>1</v>
       </c>
       <c r="F73" s="24" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G73" s="6">
         <v>129</v>
@@ -3471,25 +3465,25 @@
     </row>
     <row r="76" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H76" s="12"/>
     </row>
     <row r="77" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C77" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D77" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E77" s="7">
         <v>16</v>
       </c>
       <c r="F77" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G77" s="6">
         <v>1.31</v>
@@ -3501,19 +3495,19 @@
     </row>
     <row r="78" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="C78" t="s">
+        <v>294</v>
+      </c>
+      <c r="D78" t="s">
         <v>296</v>
       </c>
-      <c r="C78" t="s">
-        <v>295</v>
-      </c>
-      <c r="D78" t="s">
+      <c r="E78" s="7">
+        <v>1</v>
+      </c>
+      <c r="F78" t="s">
         <v>297</v>
-      </c>
-      <c r="E78" s="7">
-        <v>1</v>
-      </c>
-      <c r="F78" t="s">
-        <v>298</v>
       </c>
       <c r="G78" s="6">
         <v>18.28</v>
@@ -3525,19 +3519,19 @@
     </row>
     <row r="79" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C79" t="s">
+        <v>298</v>
+      </c>
+      <c r="D79" t="s">
+        <v>300</v>
+      </c>
+      <c r="E79" s="7">
+        <v>1</v>
+      </c>
+      <c r="F79" t="s">
         <v>299</v>
-      </c>
-      <c r="D79" t="s">
-        <v>301</v>
-      </c>
-      <c r="E79" s="7">
-        <v>1</v>
-      </c>
-      <c r="F79" t="s">
-        <v>300</v>
       </c>
       <c r="G79" s="6">
         <v>10.81</v>
@@ -3549,19 +3543,19 @@
     </row>
     <row r="80" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="C80" t="s">
+        <v>298</v>
+      </c>
+      <c r="D80" t="s">
         <v>302</v>
       </c>
-      <c r="C80" t="s">
-        <v>299</v>
-      </c>
-      <c r="D80" t="s">
+      <c r="E80" s="7">
+        <v>1</v>
+      </c>
+      <c r="F80" t="s">
         <v>303</v>
-      </c>
-      <c r="E80" s="7">
-        <v>1</v>
-      </c>
-      <c r="F80" t="s">
-        <v>304</v>
       </c>
       <c r="G80" s="6">
         <v>7.8</v>
@@ -3573,36 +3567,36 @@
     </row>
     <row r="81" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="C81" t="s">
+        <v>416</v>
+      </c>
+      <c r="D81" t="s">
+        <v>414</v>
+      </c>
+      <c r="E81">
+        <v>1</v>
+      </c>
+      <c r="F81" t="s">
         <v>415</v>
-      </c>
-      <c r="C81" t="s">
-        <v>418</v>
-      </c>
-      <c r="D81" t="s">
-        <v>416</v>
-      </c>
-      <c r="E81">
-        <v>1</v>
-      </c>
-      <c r="F81" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="C82" t="s">
         <v>316</v>
       </c>
-      <c r="C82" t="s">
+      <c r="D82" t="s">
         <v>317</v>
       </c>
-      <c r="D82" t="s">
+      <c r="E82" s="7">
+        <v>1</v>
+      </c>
+      <c r="F82" t="s">
         <v>318</v>
-      </c>
-      <c r="E82" s="7">
-        <v>1</v>
-      </c>
-      <c r="F82" t="s">
-        <v>319</v>
       </c>
       <c r="G82" s="6">
         <v>2.19</v>
@@ -3614,19 +3608,19 @@
     </row>
     <row r="83" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C83" t="s">
         <v>308</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D83" t="s">
         <v>309</v>
       </c>
-      <c r="D83" t="s">
+      <c r="E83" s="7">
+        <v>1</v>
+      </c>
+      <c r="F83" t="s">
         <v>310</v>
-      </c>
-      <c r="E83" s="7">
-        <v>1</v>
-      </c>
-      <c r="F83" t="s">
-        <v>311</v>
       </c>
       <c r="G83" s="6">
         <v>3.51</v>
@@ -3638,13 +3632,13 @@
     </row>
     <row r="84" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C84" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D84" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="E84" s="7">
         <v>16</v>
@@ -3687,16 +3681,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="B1" s="20" t="s">
         <v>193</v>
       </c>
-      <c r="B1" s="20" t="s">
-        <v>194</v>
-      </c>
       <c r="C1" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -3704,13 +3698,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -3718,13 +3712,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -3732,13 +3726,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -3746,13 +3740,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -3760,13 +3754,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -3774,13 +3768,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -3788,13 +3782,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" t="s">
         <v>202</v>
       </c>
-      <c r="C8" t="s">
-        <v>203</v>
-      </c>
       <c r="D8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -3802,13 +3796,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="C9" t="s">
         <v>204</v>
       </c>
-      <c r="C9" t="s">
-        <v>205</v>
-      </c>
       <c r="D9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -3816,13 +3810,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C10" t="s">
         <v>206</v>
       </c>
-      <c r="C10" t="s">
-        <v>207</v>
-      </c>
       <c r="D10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -3830,13 +3824,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="C11" t="s">
         <v>208</v>
       </c>
-      <c r="C11" t="s">
-        <v>209</v>
-      </c>
       <c r="D11" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -3844,13 +3838,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D12" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -3858,13 +3852,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C13" t="s">
         <v>212</v>
       </c>
-      <c r="C13" t="s">
-        <v>213</v>
-      </c>
       <c r="D13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -3872,13 +3866,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="C14" t="s">
         <v>214</v>
       </c>
-      <c r="C14" t="s">
-        <v>215</v>
-      </c>
       <c r="D14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -3886,13 +3880,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C15" t="s">
         <v>216</v>
       </c>
-      <c r="C15" t="s">
-        <v>217</v>
-      </c>
       <c r="D15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -3900,13 +3894,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="C16" t="s">
         <v>218</v>
       </c>
-      <c r="C16" t="s">
-        <v>219</v>
-      </c>
       <c r="D16" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -3914,13 +3908,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="C17" t="s">
         <v>220</v>
       </c>
-      <c r="C17" t="s">
-        <v>221</v>
-      </c>
       <c r="D17" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -3928,13 +3922,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C18" t="s">
         <v>222</v>
       </c>
-      <c r="C18" t="s">
-        <v>223</v>
-      </c>
       <c r="D18" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -3942,13 +3936,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C19" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D19" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -3956,13 +3950,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C20" t="s">
         <v>225</v>
       </c>
-      <c r="C20" t="s">
-        <v>226</v>
-      </c>
       <c r="D20" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -3970,13 +3964,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C21" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D21" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -3984,13 +3978,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C22" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D22" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -3998,13 +3992,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C23" t="s">
         <v>229</v>
       </c>
-      <c r="C23" t="s">
-        <v>230</v>
-      </c>
       <c r="D23" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -4012,13 +4006,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="C24" t="s">
         <v>231</v>
       </c>
-      <c r="C24" t="s">
-        <v>232</v>
-      </c>
       <c r="D24" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -4026,13 +4020,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C25" t="s">
         <v>233</v>
       </c>
-      <c r="C25" t="s">
-        <v>234</v>
-      </c>
       <c r="D25" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -4040,13 +4034,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C26" t="s">
         <v>235</v>
       </c>
-      <c r="C26" t="s">
-        <v>236</v>
-      </c>
       <c r="D26" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -4054,13 +4048,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C27" t="s">
         <v>237</v>
       </c>
-      <c r="C27" t="s">
-        <v>238</v>
-      </c>
       <c r="D27" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -4068,13 +4062,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="C28" t="s">
         <v>239</v>
       </c>
-      <c r="C28" t="s">
-        <v>240</v>
-      </c>
       <c r="D28" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -4082,13 +4076,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="C29" t="s">
         <v>241</v>
       </c>
-      <c r="C29" t="s">
-        <v>242</v>
-      </c>
       <c r="D29" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -4096,13 +4090,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C30" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D30" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -4110,13 +4104,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C31" t="s">
         <v>244</v>
       </c>
-      <c r="C31" t="s">
-        <v>245</v>
-      </c>
       <c r="D31" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
@@ -4124,13 +4118,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="C32" t="s">
         <v>246</v>
       </c>
-      <c r="C32" t="s">
-        <v>247</v>
-      </c>
       <c r="D32" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
@@ -4138,13 +4132,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="C33" t="s">
         <v>248</v>
       </c>
-      <c r="C33" t="s">
-        <v>249</v>
-      </c>
       <c r="D33" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -4177,387 +4171,387 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
+        <v>354</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="33" t="s">
         <v>355</v>
       </c>
-      <c r="B1" s="26" t="s">
-        <v>136</v>
-      </c>
-      <c r="C1" s="33" t="s">
+      <c r="D1" s="26" t="s">
         <v>356</v>
       </c>
-      <c r="D1" s="26" t="s">
-        <v>357</v>
-      </c>
       <c r="F1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G1" t="s">
         <v>138</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>139</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>140</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>141</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>142</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>143</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>144</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>145</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>146</v>
-      </c>
-      <c r="O1" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
+        <v>357</v>
+      </c>
+      <c r="B2" s="28" t="s">
         <v>358</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>359</v>
       </c>
       <c r="C2" s="34">
         <v>28</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C3" s="34">
         <v>1</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C4" s="35">
         <v>2</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C5" s="35">
         <v>2</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C6" s="35">
         <v>2</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C7" s="34">
         <v>1</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="32" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C8" s="35">
         <v>24</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="29" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C9" s="35">
         <v>4</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C10" s="35">
         <v>1</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C11" s="34">
         <v>3</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C12" s="34">
         <v>1</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C13" s="35">
         <v>1</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C14" s="34">
         <v>2</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A15" s="32" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C15" s="35">
         <v>16</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C16" s="34">
         <v>2</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="27" t="s">
+        <v>186</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>188</v>
+      </c>
+      <c r="C17" s="34">
+        <v>1</v>
+      </c>
+      <c r="D17" s="28" t="s">
         <v>187</v>
-      </c>
-      <c r="B17" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="C17" s="34">
-        <v>1</v>
-      </c>
-      <c r="D17" s="28" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
+        <v>158</v>
+      </c>
+      <c r="B18" s="28" t="s">
         <v>159</v>
       </c>
-      <c r="B18" s="28" t="s">
-        <v>160</v>
-      </c>
       <c r="C18" s="34">
         <v>1</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="29" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C19" s="35">
         <v>1</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>153</v>
+      </c>
+      <c r="C20" s="34">
+        <v>1</v>
+      </c>
+      <c r="D20" s="28" t="s">
         <v>152</v>
-      </c>
-      <c r="B20" s="28" t="s">
-        <v>154</v>
-      </c>
-      <c r="C20" s="34">
-        <v>1</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="B21" s="28" t="s">
         <v>165</v>
       </c>
-      <c r="B21" s="28" t="s">
-        <v>166</v>
-      </c>
       <c r="C21" s="34">
         <v>1</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="29" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C22" s="35">
         <v>1</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="B23" s="28" t="s">
         <v>161</v>
       </c>
-      <c r="B23" s="28" t="s">
-        <v>162</v>
-      </c>
       <c r="C23" s="34">
         <v>1</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C24" s="34">
         <v>1</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="B25" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="B25" s="28" t="s">
-        <v>164</v>
-      </c>
       <c r="C25" s="34">
         <v>1</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B26" s="28" t="s">
         <v>73</v>
@@ -4566,105 +4560,105 @@
         <v>1</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="29" t="s">
+        <v>184</v>
+      </c>
+      <c r="B27" s="30" t="s">
         <v>185</v>
       </c>
-      <c r="B27" s="30" t="s">
-        <v>186</v>
-      </c>
       <c r="C27" s="35">
         <v>1</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="29" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C28" s="35">
         <v>1</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="29" t="s">
+        <v>373</v>
+      </c>
+      <c r="B29" s="30" t="s">
         <v>374</v>
       </c>
-      <c r="B29" s="30" t="s">
-        <v>375</v>
-      </c>
       <c r="C29" s="35">
         <v>1</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="29" t="s">
+        <v>375</v>
+      </c>
+      <c r="B30" s="30" t="s">
         <v>376</v>
       </c>
-      <c r="B30" s="30" t="s">
-        <v>377</v>
-      </c>
       <c r="C30" s="35">
         <v>1</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="27" t="s">
+        <v>174</v>
+      </c>
+      <c r="B31" s="28" t="s">
         <v>175</v>
       </c>
-      <c r="B31" s="28" t="s">
-        <v>176</v>
-      </c>
       <c r="C31" s="34">
         <v>1</v>
       </c>
       <c r="D31" s="28" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="29" t="s">
+        <v>189</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="C32" s="35">
+        <v>1</v>
+      </c>
+      <c r="D32" s="30" t="s">
         <v>190</v>
-      </c>
-      <c r="B32" s="30" t="s">
-        <v>192</v>
-      </c>
-      <c r="C32" s="35">
-        <v>1</v>
-      </c>
-      <c r="D32" s="30" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="78" spans="6:13" x14ac:dyDescent="0.2">
       <c r="G78" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H78">
         <v>1296592</v>
       </c>
       <c r="I78" t="s">
+        <v>170</v>
+      </c>
+      <c r="J78" t="s">
         <v>171</v>
-      </c>
-      <c r="J78" t="s">
-        <v>172</v>
       </c>
       <c r="M78" t="s">
         <v>93</v>
@@ -4672,7 +4666,7 @@
     </row>
     <row r="79" spans="6:13" x14ac:dyDescent="0.2">
       <c r="F79" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G79" t="s">
         <v>73</v>
@@ -4681,17 +4675,17 @@
         <v>1462926</v>
       </c>
       <c r="I79" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="81" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K81" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="126" spans="14:14" x14ac:dyDescent="0.2">
       <c r="N126" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix PCB DRC errors and updated parts list
Updated parts list for more accurate DS3231 chip
</commit_message>
<xml_diff>
--- a/KiCad_files/MusselGapeTracker_RevI/MusselGapeTracker_RevI_parts_list.xlsx
+++ b/KiCad_files/MusselGapeTracker_RevI/MusselGapeTracker_RevI_parts_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/Documents/GitHub/MusselGapeTracker_hardware/KiCad_files/MusselGapeTracker_RevI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43077F51-7C1D-624E-9A16-CF8452D05F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93FBC69E-9C30-D341-B4F8-F65DAD3036DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1143,9 +1143,6 @@
     <t>DS3231M+TRLCT-ND</t>
   </si>
   <si>
-    <t>Real Time Clock, DS3231M+TRL  SO-16 footprint</t>
-  </si>
-  <si>
     <t>DS3231M+TRL</t>
   </si>
   <si>
@@ -1412,6 +1409,9 @@
   </si>
   <si>
     <t>WM11190CT-ND</t>
+  </si>
+  <si>
+    <t>Real Time Clock, DS3231SN#  SO-16 footprint</t>
   </si>
 </sst>
 </file>
@@ -2052,7 +2052,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="15" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -2081,7 +2081,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="J2" s="15" t="s">
         <v>337</v>
@@ -2188,13 +2188,13 @@
         <v>20</v>
       </c>
       <c r="D6" t="s">
+        <v>418</v>
+      </c>
+      <c r="E6" s="7">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
         <v>419</v>
-      </c>
-      <c r="E6" s="7">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
-        <v>420</v>
       </c>
       <c r="G6" s="6">
         <v>0.65</v>
@@ -2204,7 +2204,7 @@
         <v>0.65</v>
       </c>
       <c r="I6" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
@@ -2491,32 +2491,32 @@
     </row>
     <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>352</v>
+        <v>438</v>
       </c>
       <c r="C17" t="s">
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>353</v>
+        <v>406</v>
       </c>
       <c r="E17" s="7">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>351</v>
+        <v>407</v>
       </c>
       <c r="G17" s="6">
-        <v>12.46</v>
+        <v>17.21</v>
       </c>
       <c r="H17" s="6">
         <f t="shared" si="0"/>
-        <v>12.46</v>
+        <v>17.21</v>
       </c>
       <c r="J17" t="s">
-        <v>407</v>
+        <v>352</v>
       </c>
       <c r="K17" t="s">
-        <v>408</v>
+        <v>351</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2597,7 +2597,7 @@
         <v>3.84</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2624,7 +2624,7 @@
         <v>1.6</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2798,13 +2798,13 @@
     </row>
     <row r="28" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="40" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B28" t="s">
         <v>95</v>
       </c>
       <c r="C28" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D28" t="s">
         <v>345</v>
@@ -2823,7 +2823,7 @@
         <v>0.42</v>
       </c>
       <c r="I28" s="41" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="J28" t="s">
         <v>96</v>
@@ -2849,7 +2849,7 @@
         <v>2</v>
       </c>
       <c r="F29" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G29" s="6">
         <v>0.72</v>
@@ -2861,7 +2861,7 @@
     </row>
     <row r="30" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="40" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B30" t="s">
         <v>102</v>
@@ -2876,7 +2876,7 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G30" s="6">
         <v>2.62</v>
@@ -2886,24 +2886,24 @@
         <v>2.62</v>
       </c>
       <c r="I30" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="37" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C31" t="s">
         <v>101</v>
       </c>
       <c r="D31" t="s">
+        <v>422</v>
+      </c>
+      <c r="E31" s="7">
+        <v>1</v>
+      </c>
+      <c r="F31" t="s">
         <v>423</v>
-      </c>
-      <c r="E31" s="7">
-        <v>1</v>
-      </c>
-      <c r="F31" t="s">
-        <v>424</v>
       </c>
       <c r="G31" s="6">
         <v>1.25</v>
@@ -2913,7 +2913,7 @@
         <v>1.25</v>
       </c>
       <c r="I31" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2927,13 +2927,13 @@
         <v>93</v>
       </c>
       <c r="D32" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E32" s="7">
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="G32" s="6">
         <v>2.74</v>
@@ -2943,10 +2943,10 @@
         <v>2.74</v>
       </c>
       <c r="J32" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="K32" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3102,7 +3102,7 @@
         <v>0.16</v>
       </c>
       <c r="I38" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3129,7 +3129,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="I39" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3156,7 +3156,7 @@
         <v>1.5</v>
       </c>
       <c r="I40" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="H42" s="19">
         <f>SUM(H3:H37)</f>
-        <v>71.689999999999969</v>
+        <v>76.439999999999969</v>
       </c>
       <c r="I42" t="s">
         <v>120</v>
@@ -3188,13 +3188,13 @@
         <v>293</v>
       </c>
       <c r="D44" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E44" s="7">
         <v>72</v>
       </c>
       <c r="F44" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="G44" s="12">
         <v>0.26</v>
@@ -3204,15 +3204,15 @@
         <v>18.72</v>
       </c>
       <c r="I44" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E45" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="G45" s="42" t="s">
         <v>433</v>
-      </c>
-      <c r="G45" s="42" t="s">
-        <v>434</v>
       </c>
       <c r="H45" s="12"/>
     </row>
@@ -3224,10 +3224,10 @@
     </row>
     <row r="57" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E57" s="7">
         <v>1</v>
@@ -3245,10 +3245,10 @@
     </row>
     <row r="58" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="C58" s="23" t="s">
         <v>409</v>
-      </c>
-      <c r="C58" s="23" t="s">
-        <v>410</v>
       </c>
       <c r="E58" s="7">
         <v>16</v>
@@ -3275,7 +3275,7 @@
     </row>
     <row r="61" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C61" t="s">
         <v>319</v>
@@ -3296,7 +3296,7 @@
     </row>
     <row r="62" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C62" t="s">
         <v>319</v>
@@ -3321,13 +3321,13 @@
     </row>
     <row r="65" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E65" s="7">
+        <v>1</v>
+      </c>
+      <c r="F65" s="36" t="s">
         <v>399</v>
-      </c>
-      <c r="E65" s="7">
-        <v>1</v>
-      </c>
-      <c r="F65" s="36" t="s">
-        <v>400</v>
       </c>
       <c r="G65" s="6">
         <v>9.99</v>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="H68" s="12">
         <f>SUM(H44:H66,H3:H37)</f>
-        <v>130.45666666666665</v>
+        <v>135.20666666666668</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="20" x14ac:dyDescent="0.25">
@@ -3519,7 +3519,7 @@
     </row>
     <row r="79" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C79" t="s">
         <v>298</v>
@@ -3567,19 +3567,19 @@
     </row>
     <row r="81" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="C81" t="s">
+        <v>415</v>
+      </c>
+      <c r="D81" t="s">
         <v>413</v>
       </c>
-      <c r="C81" t="s">
-        <v>416</v>
-      </c>
-      <c r="D81" t="s">
+      <c r="E81">
+        <v>1</v>
+      </c>
+      <c r="F81" t="s">
         <v>414</v>
-      </c>
-      <c r="E81">
-        <v>1</v>
-      </c>
-      <c r="F81" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
@@ -3632,13 +3632,13 @@
     </row>
     <row r="84" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C84" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D84" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E84" s="7">
         <v>16</v>
@@ -4171,16 +4171,16 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B1" s="26" t="s">
         <v>135</v>
       </c>
       <c r="C1" s="33" t="s">
+        <v>354</v>
+      </c>
+      <c r="D1" s="26" t="s">
         <v>355</v>
-      </c>
-      <c r="D1" s="26" t="s">
-        <v>356</v>
       </c>
       <c r="F1" t="s">
         <v>137</v>
@@ -4215,16 +4215,16 @@
     </row>
     <row r="2" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
+        <v>356</v>
+      </c>
+      <c r="B2" s="28" t="s">
         <v>357</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>358</v>
       </c>
       <c r="C2" s="34">
         <v>28</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -4232,18 +4232,18 @@
         <v>321</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C3" s="34">
         <v>1</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B4" s="30" t="s">
         <v>154</v>
@@ -4252,12 +4252,12 @@
         <v>2</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>178</v>
@@ -4266,12 +4266,12 @@
         <v>2</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>178</v>
@@ -4280,7 +4280,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -4294,12 +4294,12 @@
         <v>1</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="32" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B8" s="30" t="s">
         <v>178</v>
@@ -4308,12 +4308,12 @@
         <v>24</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="29" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B9" s="30" t="s">
         <v>178</v>
@@ -4322,7 +4322,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -4336,12 +4336,12 @@
         <v>1</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B11" s="28" t="s">
         <v>178</v>
@@ -4350,7 +4350,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -4364,7 +4364,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -4378,12 +4378,12 @@
         <v>1</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B14" s="28" t="s">
         <v>148</v>
@@ -4397,7 +4397,7 @@
     </row>
     <row r="15" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A15" s="32" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B15" s="30" t="s">
         <v>157</v>
@@ -4406,12 +4406,12 @@
         <v>16</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B16" s="28" t="s">
         <v>183</v>
@@ -4448,7 +4448,7 @@
         <v>1</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -4456,7 +4456,7 @@
         <v>181</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C19" s="35">
         <v>1</v>
@@ -4490,7 +4490,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -4504,7 +4504,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -4518,12 +4518,12 @@
         <v>1</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B24" s="28" t="s">
         <v>156</v>
@@ -4546,12 +4546,12 @@
         <v>1</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B26" s="28" t="s">
         <v>73</v>
@@ -4560,7 +4560,7 @@
         <v>1</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -4574,12 +4574,12 @@
         <v>1</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="29" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B28" s="30" t="s">
         <v>150</v>
@@ -4593,30 +4593,30 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="29" t="s">
+        <v>372</v>
+      </c>
+      <c r="B29" s="30" t="s">
         <v>373</v>
       </c>
-      <c r="B29" s="30" t="s">
-        <v>374</v>
-      </c>
       <c r="C29" s="35">
         <v>1</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="29" t="s">
+        <v>374</v>
+      </c>
+      <c r="B30" s="30" t="s">
         <v>375</v>
       </c>
-      <c r="B30" s="30" t="s">
-        <v>376</v>
-      </c>
       <c r="C30" s="35">
         <v>1</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -4630,7 +4630,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="28" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>